<commit_message>
Handle automático en Excel + inicio integración Supabase pública
Tarea 1 - Handle Automático:
- Modificado import-from-excel.ts para generar handle desde título automáticamente
- Función generateHandle() convierte "Bolso Playa" → "bolso-playa"
- Variantes ahora referencian por product_title (más fácil para usuario)
- Actualizada plantilla Excel sin columna handle
- Actualizada guía de importación

Tarea 2 - Inicio integración pública:
- Creado supabase-public.ts con funciones de lectura pública
- getPublicProducts() - obtener todos los productos
- getPublicProductByHandle() - obtener producto por URL
- searchPublicProducts() - búsqueda de productos
- Transformación de datos Supabase al formato UI

Pendiente: Actualizar páginas index.tsx y [handle].tsx para usar Supabase

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/plantilla-productos.xlsx
+++ b/templates/plantilla-productos.xlsx
@@ -399,119 +399,109 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:I3"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
     <col min="4" max="4" width="50.83203125" customWidth="1"/>
-    <col min="5" max="5" width="50.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>handle</v>
+        <v>title</v>
       </c>
       <c r="B1" t="str">
-        <v>title</v>
+        <v>title_en</v>
       </c>
       <c r="C1" t="str">
-        <v>title_en</v>
+        <v>description_html</v>
       </c>
       <c r="D1" t="str">
-        <v>description_html</v>
+        <v>description_html_en</v>
       </c>
       <c r="E1" t="str">
-        <v>description_html_en</v>
+        <v>price</v>
       </c>
       <c r="F1" t="str">
-        <v>price</v>
+        <v>compare_at_price</v>
       </c>
       <c r="G1" t="str">
-        <v>compare_at_price</v>
+        <v>tags</v>
       </c>
       <c r="H1" t="str">
-        <v>tags</v>
+        <v>available_for_sale</v>
       </c>
       <c r="I1" t="str">
-        <v>available_for_sale</v>
-      </c>
-      <c r="J1" t="str">
         <v>images</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>collar-macrame-azul</v>
+        <v>Collar Macramé Azul Oceánico</v>
       </c>
       <c r="B2" t="str">
-        <v>Collar Macramé Azul Oceánico</v>
+        <v>Ocean Blue Macramé Necklace</v>
       </c>
       <c r="C2" t="str">
-        <v>Ocean Blue Macramé Necklace</v>
+        <v>&lt;p&gt;Hermoso collar hecho a mano con técnica de macramé. Cordón de algodón 100% natural teñido en tonos azules que evocan el océano.&lt;/p&gt;</v>
       </c>
       <c r="D2" t="str">
-        <v>&lt;p&gt;Hermoso collar hecho a mano con técnica de macramé. Cordón de algodón 100% natural teñido en tonos azules que evocan el océano.&lt;/p&gt;</v>
-      </c>
-      <c r="E2" t="str">
         <v>&lt;p&gt;Beautiful handmade necklace with macramé technique. 100% natural cotton cord dyed in ocean blue tones.&lt;/p&gt;</v>
       </c>
+      <c r="E2">
+        <v>45</v>
+      </c>
       <c r="F2">
-        <v>45</v>
-      </c>
-      <c r="G2">
         <v>55</v>
       </c>
+      <c r="G2" t="str">
+        <v>nuevo,collar,azul</v>
+      </c>
       <c r="H2" t="str">
-        <v>nuevo,collar,azul</v>
+        <v>TRUE</v>
       </c>
       <c r="I2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="J2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>bolso-macrame-natural</v>
+        <v>Bolso Macramé Natural</v>
       </c>
       <c r="B3" t="str">
-        <v>Bolso Macramé Natural</v>
+        <v>Natural Macramé Bag</v>
       </c>
       <c r="C3" t="str">
-        <v>Natural Macramé Bag</v>
+        <v>&lt;p&gt;Bolso artesanal de macramé en color natural. Perfecto para el día a día o la playa.&lt;/p&gt;</v>
       </c>
       <c r="D3" t="str">
-        <v>&lt;p&gt;Bolso artesanal de macramé en color natural. Perfecto para el día a día o la playa.&lt;/p&gt;</v>
-      </c>
-      <c r="E3" t="str">
         <v>&lt;p&gt;Handmade macramé bag in natural color. Perfect for everyday use or the beach.&lt;/p&gt;</v>
       </c>
-      <c r="F3">
+      <c r="E3">
         <v>89</v>
       </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
       <c r="G3" t="str">
-        <v/>
+        <v>bolso,natural</v>
       </c>
       <c r="H3" t="str">
-        <v>bolso,natural</v>
+        <v>TRUE</v>
       </c>
       <c r="I3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="J3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -520,7 +510,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L4"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
@@ -536,7 +526,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>product_handle</v>
+        <v>product_title</v>
       </c>
       <c r="B1" t="str">
         <v>largo</v>
@@ -574,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>collar-macrame-azul</v>
+        <v>Collar Macramé Azul Oceánico</v>
       </c>
       <c r="B2" t="str">
         <v>18 in</v>
@@ -612,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>collar-macrame-azul</v>
+        <v>Collar Macramé Azul Oceánico</v>
       </c>
       <c r="B3" t="str">
         <v>20 in</v>
@@ -650,7 +640,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>bolso-macrame-natural</v>
+        <v>Bolso Macramé Natural</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -695,7 +685,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A51"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
   </cols>
@@ -712,162 +702,252 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>HOJA "Productos":</v>
+        <v>¡IMPORTANTE! El "handle" (URL del producto) se genera AUTOMÁTICAMENTE desde el título.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>- handle: Identificador único para la URL (solo letras minúsculas, números y guiones). Ej: collar-macrame-azul</v>
+        <v>Ejemplo: "Bolso Playa Macramé" → bolso-playa-macrame</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>- title: Nombre del producto en español (requerido)</v>
+        <v>No necesitas crear handles manualmente.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>- title_en: Nombre del producto en inglés (opcional)</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>- description_html: Descripción en español, puede incluir HTML básico como &lt;p&gt;, &lt;b&gt;, &lt;ul&gt;</v>
+        <v>═══════════════════════════════════════════════════════════════════════</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>- description_html_en: Descripción en inglés (opcional)</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>- price: Precio en USD (número decimal). Ej: 45.00</v>
+        <v>HOJA "Productos":</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>- compare_at_price: Precio original si hay descuento (dejar vacío si no hay descuento)</v>
+        <v>- title: Nombre del producto en español (REQUERIDO)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>- tags: Etiquetas separadas por coma. Ej: nuevo,collar,azul</v>
+        <v>- title_en: Nombre del producto en inglés (opcional, para clientes que vean la web en inglés)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>- available_for_sale: TRUE si está disponible, FALSE si no</v>
+        <v>- description_html: Descripción en español, puede incluir HTML básico como &lt;p&gt;, &lt;b&gt;, &lt;ul&gt;</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>- images: URLs de imágenes separadas por | (pipe). Ej: url1|url2|url3</v>
+        <v>- description_html_en: Descripción en inglés (opcional)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v/>
+        <v>- price: Precio en USD (número decimal). Ej: 45.00</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>HOJA "Variantes":</v>
+        <v>- compare_at_price: Precio original si hay descuento (dejar vacío si no hay descuento)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>- product_handle: Handle del producto padre (debe existir en hoja Productos)</v>
+        <v>- tags: Etiquetas separadas por coma. Ej: nuevo,collar,azul</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>- largo: Opciones válidas: 16 in, 18 in, 20 in, 22 in, 24 in (dejar vacío si no aplica)</v>
+        <v>- available_for_sale: TRUE si está disponible, FALSE si no</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>- grosor: Opciones válidas: 1.5mm, 3mm, 5mm, 9mm</v>
+        <v>- images: URLs de imágenes separadas por | (pipe). Ej: url1|url2|url3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>- material_cordon: Algodón, Algodón encerado, Algodón reciclado, Nylon, Poliéster</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>- material_accesorios: Plata 925, Latón, Cobre, Bronce, Piedra natural, Cristal, Madera, Cerámica</v>
+        <v>═══════════════════════════════════════════════════════════════════════</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>- color_primario: Natural, Blanco, Negro, Gris, Beige, Marrón, Coral, Rosa, Rojo, Naranja, Amarillo, Mostaza, Verde, Verde musgo, Azul, Celeste, Azul marino, Turquesa, Morado, Dorado, Plateado</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>- color_secundario: Mismo listado que color_primario (opcional)</v>
+        <v>HOJA "Variantes":</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>- price: Precio de esta variante en USD</v>
+        <v>- product_title: TÍTULO EXACTO del producto (copia y pega de la hoja Productos)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>- compare_at_price: Precio original si hay descuento</v>
+        <v>- largo: Opciones válidas: 16 in, 18 in, 20 in, 22 in, 24 in (dejar vacío si no aplica)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>- stock: Cantidad disponible (número entero)</v>
+        <v>- grosor: Opciones válidas: 1.5mm, 3mm, 5mm, 9mm</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>- available: TRUE si está disponible, FALSE si no</v>
+        <v>- material_cordon: Algodón, Algodón encerado, Algodón reciclado, Nylon, Poliéster</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>- image: URL de imagen específica de esta variante (opcional)</v>
+        <v>- material_accesorios: Plata 925, Latón, Cobre, Bronce, Piedra natural, Cristal, Madera, Cerámica</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v/>
+        <v>- color_primario: Natural, Blanco, Negro, Gris, Beige, Marrón, Coral, Rosa, Rojo, Naranja, Amarillo, Mostaza, Verde, Verde musgo, Azul, Celeste, Azul marino, Turquesa, Morado, Dorado, Plateado</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>NOTAS IMPORTANTES:</v>
+        <v>- color_secundario: Mismo listado que color_primario (opcional)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>- Cada producto debe tener al menos una variante</v>
+        <v>- price: Precio de esta variante en USD</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>- El handle de producto debe ser único</v>
+        <v>- compare_at_price: Precio original si hay descuento</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>- Los campos marcados como requeridos no pueden estar vacíos</v>
+        <v>- stock: Cantidad disponible (número entero)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
+        <v>- available: TRUE si está disponible, FALSE si no</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>- image: URL de imagen específica de esta variante (opcional)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>═══════════════════════════════════════════════════════════════════════</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>NOTAS IMPORTANTES:</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>- Cada producto debe tener al menos una variante</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>- El título de producto debe ser ÚNICO (no repitas títulos)</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>- En variantes, el product_title debe coincidir EXACTAMENTE con el título en Productos</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>- Los campos marcados como REQUERIDO no pueden estar vacíos</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
         <v>- Para las imágenes, primero súbelas al panel admin y copia las URLs</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>═══════════════════════════════════════════════════════════════════════</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>FLUJO RECOMENDADO:</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>1. Llena primero la hoja "Productos" con títulos y descripciones</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>2. Luego llena "Variantes", copiando los títulos exactos</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>3. Ejecuta: npm run import:dry ./plantilla-productos.xlsx  (para verificar)</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>4. Si no hay errores: npm run import:products ./plantilla-productos.xlsx</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>